<commit_message>
create new contact ,customer,event files
</commit_message>
<xml_diff>
--- a/Utilities/TestData/Customer.xlsx
+++ b/Utilities/TestData/Customer.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9F0764F-945F-4FAD-89C7-08FE1F72FF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{592D6B02-DCD0-44CA-8052-3F8317CD1D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
   <si>
     <t>FieldName</t>
   </si>
@@ -60,7 +60,7 @@
     <t>VHM</t>
   </si>
   <si>
-    <t>yes</t>
+    <t>No</t>
   </si>
   <si>
     <t>Customer Name</t>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>International Address</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -169,12 +166,12 @@
     <t>Ecatering Business Unit</t>
   </si>
   <si>
+    <t>Social</t>
+  </si>
+  <si>
     <t>Business Units</t>
   </si>
   <si>
-    <t>Social</t>
-  </si>
-  <si>
     <t>Tax ID</t>
   </si>
   <si>
@@ -185,6 +182,9 @@
   </si>
   <si>
     <t>Mailing List</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
   <si>
     <t>Referral Type</t>
@@ -660,36 +660,36 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
         <v>21</v>
-      </c>
-      <c r="B13" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="s">
         <v>23</v>
-      </c>
-      <c r="B14" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -697,23 +697,23 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
         <v>26</v>
-      </c>
-      <c r="B16" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
         <v>28</v>
-      </c>
-      <c r="B17" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18">
         <v>12345</v>
@@ -721,12 +721,12 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20">
         <v>96323456</v>
@@ -734,7 +734,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -742,7 +742,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -750,7 +750,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B23">
         <v>111</v>
@@ -758,7 +758,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -766,7 +766,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B25">
         <v>11</v>
@@ -774,15 +774,15 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" t="s">
         <v>38</v>
-      </c>
-      <c r="B26" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B27">
         <v>111</v>
@@ -790,15 +790,15 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29">
         <v>1</v>
@@ -806,7 +806,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B30" s="3">
         <v>46043</v>
@@ -814,6 +814,9 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" t="s">
         <v>44</v>
       </c>
     </row>
@@ -822,12 +825,12 @@
         <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B33">
         <v>1</v>
@@ -835,7 +838,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B34">
         <v>12</v>
@@ -843,7 +846,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B35">
         <v>11</v>
@@ -851,10 +854,10 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" t="s">
         <v>50</v>
-      </c>
-      <c r="B36" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -870,7 +873,7 @@
         <v>53</v>
       </c>
       <c r="B38" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
event work flow date and contact pending
</commit_message>
<xml_diff>
--- a/Utilities/TestData/Customer.xlsx
+++ b/Utilities/TestData/Customer.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B00106F-47E4-4379-BFD3-6BA9E709ED51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="96">
   <si>
     <t>FieldName</t>
   </si>
@@ -197,63 +198,66 @@
     <t>Tax Exempt</t>
   </si>
   <si>
-    <t xml:space="preserve">Business Unit </t>
+    <t>Business Unit</t>
   </si>
   <si>
     <t>Will Call</t>
   </si>
   <si>
-    <t xml:space="preserve">Event Manager </t>
+    <t>Event Manager</t>
+  </si>
+  <si>
+    <t>Alejos , Diana</t>
+  </si>
+  <si>
+    <t>Event Type</t>
+  </si>
+  <si>
+    <t>Buffet Lunch</t>
+  </si>
+  <si>
+    <t>Platter Type</t>
+  </si>
+  <si>
+    <t>equipment</t>
+  </si>
+  <si>
+    <t>First Call Time</t>
+  </si>
+  <si>
+    <t>Revenue Stream</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>360 Live Media</t>
+  </si>
+  <si>
+    <t>Begin Time</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>abcd</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>Taiwan</t>
+  </si>
+  <si>
+    <t>Billing Customer</t>
+  </si>
+  <si>
+    <t>Account Executive</t>
   </si>
   <si>
     <t>Aarevalo , Yudi</t>
   </si>
   <si>
-    <t>Event Type</t>
-  </si>
-  <si>
-    <t>Buffet Lunch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First Call Time </t>
-  </si>
-  <si>
-    <t>Revenue Stream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Begin Time </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status </t>
-  </si>
-  <si>
-    <t>abcd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">County </t>
-  </si>
-  <si>
-    <t>Taiwan</t>
-  </si>
-  <si>
-    <t>Billing Customer</t>
-  </si>
-  <si>
-    <t>Platter Type</t>
-  </si>
-  <si>
-    <t>equipment</t>
-  </si>
-  <si>
-    <t>Account Executive</t>
-  </si>
-  <si>
-    <t>sam</t>
-  </si>
-  <si>
     <t>End Time</t>
   </si>
   <si>
@@ -269,16 +273,16 @@
     <t>New</t>
   </si>
   <si>
-    <t xml:space="preserve">Event Theme </t>
+    <t>Event Theme</t>
   </si>
   <si>
     <t>Adult Count</t>
   </si>
   <si>
-    <t xml:space="preserve">Staff Count </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated $/Person </t>
+    <t>Staff Count</t>
+  </si>
+  <si>
+    <t>Estimated $/Person</t>
   </si>
   <si>
     <t>Band Count</t>
@@ -287,55 +291,34 @@
     <t>Kids Count</t>
   </si>
   <si>
-    <t xml:space="preserve">Misc Count </t>
+    <t>Misc Count</t>
   </si>
   <si>
     <t>Contact Name</t>
   </si>
   <si>
-    <t xml:space="preserve">Zip </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suite </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrance </t>
-  </si>
-  <si>
-    <t xml:space="preserve">State </t>
+    <t>test contact</t>
   </si>
   <si>
     <t>VA</t>
   </si>
   <si>
-    <t xml:space="preserve">City </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name </t>
+    <t>Name</t>
   </si>
   <si>
     <t>test John</t>
   </si>
   <si>
-    <t xml:space="preserve">Work Phone </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email </t>
+    <t>Work Phone</t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
   <si>
     <t>test@gmail.com</t>
   </si>
   <si>
     <t>Home Phone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fax </t>
-  </si>
-  <si>
-    <t>test naame</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments </t>
   </si>
   <si>
     <t>test comments</t>
@@ -344,8 +327,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -383,6 +366,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -405,7 +394,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -415,6 +404,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -476,7 +467,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -528,7 +519,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -722,14 +713,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1038,7 +1029,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1055,7 +1046,7 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>54</v>
       </c>
       <c r="B2" t="s">
@@ -1080,93 +1071,101 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>60</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>64</v>
+      </c>
+      <c r="B8" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>63</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="B9" s="7"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>73</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="B15" s="8"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1179,7 +1178,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -1187,7 +1186,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21">
         <v>3</v>
@@ -1195,7 +1194,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B22">
         <v>4</v>
@@ -1203,7 +1202,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B23">
         <v>5</v>
@@ -1211,7 +1210,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B24">
         <v>6</v>
@@ -1219,7 +1218,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B25">
         <v>7</v>
@@ -1227,12 +1226,15 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>85</v>
+        <v>86</v>
+      </c>
+      <c r="B26" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="B27">
         <v>12345</v>
@@ -1240,7 +1242,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="B28">
         <v>1</v>
@@ -1248,7 +1250,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="B29">
         <v>2</v>
@@ -1256,10 +1258,10 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -1285,7 +1287,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="B34" t="s">
         <v>26</v>
@@ -1293,15 +1295,15 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B36">
         <v>456776543456</v>
@@ -1309,15 +1311,15 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B38">
         <v>876543456</v>
@@ -1325,26 +1327,26 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>32</v>
       </c>
       <c r="B39">
         <v>12345</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="1" t="s">
-        <v>92</v>
+      <c r="A40" t="s">
+        <v>89</v>
       </c>
       <c r="B40" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -1357,14 +1359,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B37" r:id="rId1"/>
+    <hyperlink ref="B37" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F38"/>
   <sheetFormatPr defaultColWidth="16.140625" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>